<commit_message>
ajusta inventario e equivalencias historicas
</commit_message>
<xml_diff>
--- a/data/reference/equivalencias_historicas.xlsx
+++ b/data/reference/equivalencias_historicas.xlsx
@@ -1,31 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udesc-my.sharepoint.com/personal/06376528945_udesc_br/Documents/Arquivo Permanente/sri_udesc_cct/data/reference/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_CB8642695D2F8E1ED8920972EDA4D343C38E1B5F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE8EBD4A-F2F1-487F-82CC-3041E9CE9799}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1485" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>termo_historico</t>
   </si>
@@ -38,45 +27,12 @@
   <si>
     <t>observacao</t>
   </si>
-  <si>
-    <t>PTI</t>
-  </si>
-  <si>
-    <t>Plano de Trabalho Individual</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>Sigla histórica</t>
-  </si>
-  <si>
-    <t>Ficha Escolar</t>
-  </si>
-  <si>
-    <t>Histórico Escolar de Aluno de Curso de Graduação</t>
-  </si>
-  <si>
-    <t>Nome antigo</t>
-  </si>
-  <si>
-    <t>Plano Individual de Trabalho</t>
-  </si>
-  <si>
-    <t>Denominação antiga</t>
-  </si>
-  <si>
-    <t>CI</t>
-  </si>
-  <si>
-    <t>Comunicação Interna</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,64 +40,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F5F5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFE6E6E6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFE6E6E6"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFE6E6E6"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFE6E6E6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFE6E6E6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFE6E6E6"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -150,36 +61,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -221,7 +115,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -253,27 +147,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -305,24 +181,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -498,88 +356,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>